<commit_message>
feat(production): complete institutional autopilot pipeline, live sync daemon, 1:20 mentoring, and zero-latency roster
</commit_message>
<xml_diff>
--- a/reports/Contest_Combined_2026-08-22.xlsx
+++ b/reports/Contest_Combined_2026-08-22.xlsx
@@ -1172,7 +1172,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>bharani05flow</t>
+          <t>Bharani05flow</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1388,7 +1388,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>nivetha-06</t>
+          <t>Nivetha-06</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1442,7 +1442,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>leenaperiyasamy</t>
+          <t>Leenaperiyasamy</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>thariq2625</t>
+          <t>Thariq2625</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -2792,7 +2792,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>sathyanarayanan_11062006</t>
+          <t>Sathyanarayanan_11062006</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -4412,7 +4412,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>divyabharathi01</t>
+          <t>Divyabharathi01</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
@@ -7490,7 +7490,7 @@
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>Rohan_19</t>
+          <t>rohan_19</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
@@ -17156,7 +17156,7 @@
       </c>
       <c r="G310" t="inlineStr">
         <is>
-          <t>Ratheesh_123</t>
+          <t>RATHEESH_123</t>
         </is>
       </c>
       <c r="H310" t="inlineStr">
@@ -27362,7 +27362,7 @@
       </c>
       <c r="G499" t="inlineStr">
         <is>
-          <t>Sanjayece</t>
+          <t>sanjayece</t>
         </is>
       </c>
       <c r="H499" t="inlineStr">
@@ -32222,7 +32222,7 @@
       </c>
       <c r="G589" t="inlineStr">
         <is>
-          <t>puja2007_03</t>
+          <t>Puja2007_03</t>
         </is>
       </c>
       <c r="H589" t="inlineStr">
@@ -32492,7 +32492,7 @@
       </c>
       <c r="G594" t="inlineStr">
         <is>
-          <t>Roshh_07</t>
+          <t>roshh_07</t>
         </is>
       </c>
       <c r="H594" t="inlineStr">
@@ -33788,7 +33788,7 @@
       </c>
       <c r="G618" t="inlineStr">
         <is>
-          <t>swathi_28_11_2006</t>
+          <t>Swathi_28_11_2006</t>
         </is>
       </c>
       <c r="H618" t="inlineStr">
@@ -36326,7 +36326,7 @@
       </c>
       <c r="G665" t="inlineStr">
         <is>
-          <t>Karthik_16</t>
+          <t>karthik_16</t>
         </is>
       </c>
       <c r="H665" t="inlineStr">
@@ -36650,7 +36650,7 @@
       </c>
       <c r="G671" t="inlineStr">
         <is>
-          <t>kishor</t>
+          <t>Kishor</t>
         </is>
       </c>
       <c r="H671" t="inlineStr">
@@ -38648,7 +38648,7 @@
       </c>
       <c r="G708" t="inlineStr">
         <is>
-          <t>santhiya</t>
+          <t>Santhiya</t>
         </is>
       </c>
       <c r="H708" t="inlineStr">
@@ -47288,7 +47288,7 @@
       </c>
       <c r="G868" t="inlineStr">
         <is>
-          <t>KARTHIKXK</t>
+          <t>KARTHIKxK</t>
         </is>
       </c>
       <c r="H868" t="inlineStr">
@@ -51770,7 +51770,7 @@
       </c>
       <c r="G951" t="inlineStr">
         <is>
-          <t>pugalenthi_m</t>
+          <t>pugalenthi_M</t>
         </is>
       </c>
       <c r="H951" t="inlineStr">
@@ -57980,7 +57980,7 @@
       </c>
       <c r="G1066" t="inlineStr">
         <is>
-          <t>ROHITH_P</t>
+          <t>Rohith_P</t>
         </is>
       </c>
       <c r="H1066" t="inlineStr">
@@ -58574,7 +58574,7 @@
       </c>
       <c r="G1077" t="inlineStr">
         <is>
-          <t>SMITHA_M</t>
+          <t>Smitha_M</t>
         </is>
       </c>
       <c r="H1077" t="inlineStr">
@@ -61706,7 +61706,7 @@
       </c>
       <c r="G1135" t="inlineStr">
         <is>
-          <t>KLITHES</t>
+          <t>klithes</t>
         </is>
       </c>
       <c r="H1135" t="inlineStr">
@@ -62894,7 +62894,7 @@
       </c>
       <c r="G1157" t="inlineStr">
         <is>
-          <t>Pradheesh_k18</t>
+          <t>pradheesh_k18</t>
         </is>
       </c>
       <c r="H1157" t="inlineStr">
@@ -63650,7 +63650,7 @@
       </c>
       <c r="G1171" t="inlineStr">
         <is>
-          <t>samithra_13</t>
+          <t>Samithra_13</t>
         </is>
       </c>
       <c r="H1171" t="inlineStr">
@@ -63704,7 +63704,7 @@
       </c>
       <c r="G1172" t="inlineStr">
         <is>
-          <t>santhosh_007</t>
+          <t>Santhosh_007</t>
         </is>
       </c>
       <c r="H1172" t="inlineStr">
@@ -64244,7 +64244,7 @@
       </c>
       <c r="G1182" t="inlineStr">
         <is>
-          <t>srikanth_24_2007</t>
+          <t>Srikanth_24_2007</t>
         </is>
       </c>
       <c r="H1182" t="inlineStr">
@@ -64514,7 +64514,7 @@
       </c>
       <c r="G1187" t="inlineStr">
         <is>
-          <t>Surya-s-r</t>
+          <t>surya-s-r</t>
         </is>
       </c>
       <c r="H1187" t="inlineStr">
@@ -64676,7 +64676,7 @@
       </c>
       <c r="G1190" t="inlineStr">
         <is>
-          <t>Tamil_2805</t>
+          <t>tamil_2805</t>
         </is>
       </c>
       <c r="H1190" t="inlineStr">
@@ -66944,7 +66944,7 @@
       </c>
       <c r="G1232" t="inlineStr">
         <is>
-          <t>dhilipKumar_s</t>
+          <t>dhilipkumar_s</t>
         </is>
       </c>
       <c r="H1232" t="inlineStr">
@@ -69482,7 +69482,7 @@
       </c>
       <c r="G1279" t="inlineStr">
         <is>
-          <t>Akshaya_07_</t>
+          <t>akshaya_07_</t>
         </is>
       </c>
       <c r="H1279" t="inlineStr">

</xml_diff>

<commit_message>
feat(contest): finalize Weekly Contest 516 with 53 verified solvers and lock immutable snapshot
</commit_message>
<xml_diff>
--- a/reports/Contest_Combined_2026-08-22.xlsx
+++ b/reports/Contest_Combined_2026-08-22.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1396"/>
+  <dimension ref="A1:L1473"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -75823,6 +75823,4164 @@
         <v>0</v>
       </c>
     </row>
+    <row r="1397">
+      <c r="A1397" t="n">
+        <v>1396</v>
+      </c>
+      <c r="B1397" t="inlineStr">
+        <is>
+          <t>732223CC001</t>
+        </is>
+      </c>
+      <c r="C1397" t="inlineStr">
+        <is>
+          <t>AATHAVAN T</t>
+        </is>
+      </c>
+      <c r="D1397" t="inlineStr">
+        <is>
+          <t>CSE(CS)</t>
+        </is>
+      </c>
+      <c r="E1397" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="F1397" t="inlineStr">
+        <is>
+          <t>2023 - 2027</t>
+        </is>
+      </c>
+      <c r="G1397" t="inlineStr">
+        <is>
+          <t>aathavanthiyakeswaran</t>
+        </is>
+      </c>
+      <c r="H1397" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1397" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1397" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1397" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1397" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1398">
+      <c r="A1398" t="n">
+        <v>1397</v>
+      </c>
+      <c r="B1398" t="inlineStr">
+        <is>
+          <t>732223CC002</t>
+        </is>
+      </c>
+      <c r="C1398" t="inlineStr">
+        <is>
+          <t>S.ABIRAMI</t>
+        </is>
+      </c>
+      <c r="D1398" t="inlineStr">
+        <is>
+          <t>CSE(CS)</t>
+        </is>
+      </c>
+      <c r="E1398" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="F1398" t="inlineStr">
+        <is>
+          <t>2023 - 2027</t>
+        </is>
+      </c>
+      <c r="G1398" t="inlineStr">
+        <is>
+          <t>slrlj6cnjl</t>
+        </is>
+      </c>
+      <c r="H1398" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1398" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1398" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1398" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1398" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1399">
+      <c r="A1399" t="n">
+        <v>1398</v>
+      </c>
+      <c r="B1399" t="inlineStr">
+        <is>
+          <t>732223CC003</t>
+        </is>
+      </c>
+      <c r="C1399" t="inlineStr">
+        <is>
+          <t>ASWIN P</t>
+        </is>
+      </c>
+      <c r="D1399" t="inlineStr">
+        <is>
+          <t>CSE(CS)</t>
+        </is>
+      </c>
+      <c r="E1399" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="F1399" t="inlineStr">
+        <is>
+          <t>2023 - 2027</t>
+        </is>
+      </c>
+      <c r="G1399" t="inlineStr">
+        <is>
+          <t>aswinkasin</t>
+        </is>
+      </c>
+      <c r="H1399" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1399" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1399" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1399" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1399" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1400">
+      <c r="A1400" t="n">
+        <v>1399</v>
+      </c>
+      <c r="B1400" t="inlineStr">
+        <is>
+          <t>732223CC005</t>
+        </is>
+      </c>
+      <c r="C1400" t="inlineStr">
+        <is>
+          <t>BHARATH I</t>
+        </is>
+      </c>
+      <c r="D1400" t="inlineStr">
+        <is>
+          <t>CSE(CS)</t>
+        </is>
+      </c>
+      <c r="E1400" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="F1400" t="inlineStr">
+        <is>
+          <t>2023 - 2027</t>
+        </is>
+      </c>
+      <c r="G1400" t="inlineStr">
+        <is>
+          <t>bharath_77</t>
+        </is>
+      </c>
+      <c r="H1400" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1400" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1400" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1400" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1400" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1401">
+      <c r="A1401" t="n">
+        <v>1400</v>
+      </c>
+      <c r="B1401" t="inlineStr">
+        <is>
+          <t>732223CC007</t>
+        </is>
+      </c>
+      <c r="C1401" t="inlineStr">
+        <is>
+          <t>DEEPADHARSHINI C</t>
+        </is>
+      </c>
+      <c r="D1401" t="inlineStr">
+        <is>
+          <t>CSE(CS)</t>
+        </is>
+      </c>
+      <c r="E1401" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="F1401" t="inlineStr">
+        <is>
+          <t>2023 - 2027</t>
+        </is>
+      </c>
+      <c r="G1401" t="inlineStr">
+        <is>
+          <t>deepadharshini_10</t>
+        </is>
+      </c>
+      <c r="H1401" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1401" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1401" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1401" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1401" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1402">
+      <c r="A1402" t="n">
+        <v>1401</v>
+      </c>
+      <c r="B1402" t="inlineStr">
+        <is>
+          <t>732223CC009</t>
+        </is>
+      </c>
+      <c r="C1402" t="inlineStr">
+        <is>
+          <t>DEEPAKKUMAR E</t>
+        </is>
+      </c>
+      <c r="D1402" t="inlineStr">
+        <is>
+          <t>CSE(CS)</t>
+        </is>
+      </c>
+      <c r="E1402" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="F1402" t="inlineStr">
+        <is>
+          <t>2023 - 2027</t>
+        </is>
+      </c>
+      <c r="G1402" t="inlineStr">
+        <is>
+          <t>deepak1524</t>
+        </is>
+      </c>
+      <c r="H1402" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1402" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1402" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1402" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1402" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1403">
+      <c r="A1403" t="n">
+        <v>1402</v>
+      </c>
+      <c r="B1403" t="inlineStr">
+        <is>
+          <t>732223CC010</t>
+        </is>
+      </c>
+      <c r="C1403" t="inlineStr">
+        <is>
+          <t>DEEPAKKUMAR M</t>
+        </is>
+      </c>
+      <c r="D1403" t="inlineStr">
+        <is>
+          <t>CSE(CS)</t>
+        </is>
+      </c>
+      <c r="E1403" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="F1403" t="inlineStr">
+        <is>
+          <t>2023 - 2027</t>
+        </is>
+      </c>
+      <c r="G1403" t="inlineStr">
+        <is>
+          <t>deepak2612</t>
+        </is>
+      </c>
+      <c r="H1403" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1403" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1403" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1403" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1403" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1404">
+      <c r="A1404" t="n">
+        <v>1403</v>
+      </c>
+      <c r="B1404" t="inlineStr">
+        <is>
+          <t>732223CC013</t>
+        </is>
+      </c>
+      <c r="C1404" t="inlineStr">
+        <is>
+          <t>ENIYAVAN R</t>
+        </is>
+      </c>
+      <c r="D1404" t="inlineStr">
+        <is>
+          <t>CSE(CS)</t>
+        </is>
+      </c>
+      <c r="E1404" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="F1404" t="inlineStr">
+        <is>
+          <t>2023 - 2027</t>
+        </is>
+      </c>
+      <c r="G1404" t="inlineStr">
+        <is>
+          <t>eniyavan_r</t>
+        </is>
+      </c>
+      <c r="H1404" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1404" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1404" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1404" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1404" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1405">
+      <c r="A1405" t="n">
+        <v>1404</v>
+      </c>
+      <c r="B1405" t="inlineStr">
+        <is>
+          <t>732223CC017</t>
+        </is>
+      </c>
+      <c r="C1405" t="inlineStr">
+        <is>
+          <t>JANARANSHINI P</t>
+        </is>
+      </c>
+      <c r="D1405" t="inlineStr">
+        <is>
+          <t>CSE(CS)</t>
+        </is>
+      </c>
+      <c r="E1405" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="F1405" t="inlineStr">
+        <is>
+          <t>2023 - 2027</t>
+        </is>
+      </c>
+      <c r="G1405" t="inlineStr">
+        <is>
+          <t>janaranshini_17</t>
+        </is>
+      </c>
+      <c r="H1405" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1405" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1405" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1405" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1405" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1406">
+      <c r="A1406" t="n">
+        <v>1405</v>
+      </c>
+      <c r="B1406" t="inlineStr">
+        <is>
+          <t>732223CC020</t>
+        </is>
+      </c>
+      <c r="C1406" t="inlineStr">
+        <is>
+          <t>KANISHAA.K.S</t>
+        </is>
+      </c>
+      <c r="D1406" t="inlineStr">
+        <is>
+          <t>CSE(CS)</t>
+        </is>
+      </c>
+      <c r="E1406" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="F1406" t="inlineStr">
+        <is>
+          <t>2023 - 2027</t>
+        </is>
+      </c>
+      <c r="G1406" t="inlineStr">
+        <is>
+          <t>kani_shan</t>
+        </is>
+      </c>
+      <c r="H1406" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1406" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1406" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1406" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1406" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1407">
+      <c r="A1407" t="n">
+        <v>1406</v>
+      </c>
+      <c r="B1407" t="inlineStr">
+        <is>
+          <t>732223CC021</t>
+        </is>
+      </c>
+      <c r="C1407" t="inlineStr">
+        <is>
+          <t>KANISKA N J</t>
+        </is>
+      </c>
+      <c r="D1407" t="inlineStr">
+        <is>
+          <t>CSE(CS)</t>
+        </is>
+      </c>
+      <c r="E1407" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="F1407" t="inlineStr">
+        <is>
+          <t>2023 - 2027</t>
+        </is>
+      </c>
+      <c r="G1407" t="inlineStr">
+        <is>
+          <t>ka_nizzu29</t>
+        </is>
+      </c>
+      <c r="H1407" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1407" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1407" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1407" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1407" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1408">
+      <c r="A1408" t="n">
+        <v>1407</v>
+      </c>
+      <c r="B1408" t="inlineStr">
+        <is>
+          <t>732223CC023</t>
+        </is>
+      </c>
+      <c r="C1408" t="inlineStr">
+        <is>
+          <t>KAVINRAJAN K</t>
+        </is>
+      </c>
+      <c r="D1408" t="inlineStr">
+        <is>
+          <t>CSE(CS)</t>
+        </is>
+      </c>
+      <c r="E1408" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="F1408" t="inlineStr">
+        <is>
+          <t>2023 - 2027</t>
+        </is>
+      </c>
+      <c r="G1408" t="inlineStr">
+        <is>
+          <t>kavinrajan</t>
+        </is>
+      </c>
+      <c r="H1408" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1408" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1408" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1408" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1408" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1409">
+      <c r="A1409" t="n">
+        <v>1408</v>
+      </c>
+      <c r="B1409" t="inlineStr">
+        <is>
+          <t>732223CC025</t>
+        </is>
+      </c>
+      <c r="C1409" t="inlineStr">
+        <is>
+          <t>KEERTHANA B</t>
+        </is>
+      </c>
+      <c r="D1409" t="inlineStr">
+        <is>
+          <t>CSE(CS)</t>
+        </is>
+      </c>
+      <c r="E1409" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="F1409" t="inlineStr">
+        <is>
+          <t>2023 - 2027</t>
+        </is>
+      </c>
+      <c r="G1409" t="inlineStr">
+        <is>
+          <t>keerthu-2005</t>
+        </is>
+      </c>
+      <c r="H1409" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1409" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1409" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1409" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1409" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1410">
+      <c r="A1410" t="n">
+        <v>1409</v>
+      </c>
+      <c r="B1410" t="inlineStr">
+        <is>
+          <t>732223CC031</t>
+        </is>
+      </c>
+      <c r="C1410" t="inlineStr">
+        <is>
+          <t>MOWNAVARTHINI A L</t>
+        </is>
+      </c>
+      <c r="D1410" t="inlineStr">
+        <is>
+          <t>CSE(CS)</t>
+        </is>
+      </c>
+      <c r="E1410" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="F1410" t="inlineStr">
+        <is>
+          <t>2023 - 2027</t>
+        </is>
+      </c>
+      <c r="G1410" t="inlineStr">
+        <is>
+          <t>mowna_14</t>
+        </is>
+      </c>
+      <c r="H1410" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1410" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1410" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1410" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1410" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1411">
+      <c r="A1411" t="n">
+        <v>1410</v>
+      </c>
+      <c r="B1411" t="inlineStr">
+        <is>
+          <t>732223CC038</t>
+        </is>
+      </c>
+      <c r="C1411" t="inlineStr">
+        <is>
+          <t>PRAVEEN KUMAR J</t>
+        </is>
+      </c>
+      <c r="D1411" t="inlineStr">
+        <is>
+          <t>CSE(CS)</t>
+        </is>
+      </c>
+      <c r="E1411" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="F1411" t="inlineStr">
+        <is>
+          <t>2023 - 2027</t>
+        </is>
+      </c>
+      <c r="G1411" t="inlineStr">
+        <is>
+          <t>praveen360</t>
+        </is>
+      </c>
+      <c r="H1411" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1411" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1411" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1411" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1411" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1412">
+      <c r="A1412" t="n">
+        <v>1411</v>
+      </c>
+      <c r="B1412" t="inlineStr">
+        <is>
+          <t>732223CC039</t>
+        </is>
+      </c>
+      <c r="C1412" t="inlineStr">
+        <is>
+          <t>PRAVEEN VENKATESH A V</t>
+        </is>
+      </c>
+      <c r="D1412" t="inlineStr">
+        <is>
+          <t>CSE(CS)</t>
+        </is>
+      </c>
+      <c r="E1412" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="F1412" t="inlineStr">
+        <is>
+          <t>2023 - 2027</t>
+        </is>
+      </c>
+      <c r="G1412" t="inlineStr">
+        <is>
+          <t>pravexn</t>
+        </is>
+      </c>
+      <c r="H1412" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1412" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1412" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1412" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1412" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1413">
+      <c r="A1413" t="n">
+        <v>1412</v>
+      </c>
+      <c r="B1413" t="inlineStr">
+        <is>
+          <t>732223CC042</t>
+        </is>
+      </c>
+      <c r="C1413" t="inlineStr">
+        <is>
+          <t>PRIYADHARSHINI K</t>
+        </is>
+      </c>
+      <c r="D1413" t="inlineStr">
+        <is>
+          <t>CSE(CS)</t>
+        </is>
+      </c>
+      <c r="E1413" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="F1413" t="inlineStr">
+        <is>
+          <t>2023 - 2027</t>
+        </is>
+      </c>
+      <c r="G1413" t="inlineStr">
+        <is>
+          <t>dhars_02</t>
+        </is>
+      </c>
+      <c r="H1413" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1413" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1413" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1413" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1413" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1414">
+      <c r="A1414" t="n">
+        <v>1413</v>
+      </c>
+      <c r="B1414" t="inlineStr">
+        <is>
+          <t>732223CC043</t>
+        </is>
+      </c>
+      <c r="C1414" t="inlineStr">
+        <is>
+          <t>RAGAVAN S</t>
+        </is>
+      </c>
+      <c r="D1414" t="inlineStr">
+        <is>
+          <t>CSE(CS)</t>
+        </is>
+      </c>
+      <c r="E1414" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="F1414" t="inlineStr">
+        <is>
+          <t>2023 - 2027</t>
+        </is>
+      </c>
+      <c r="G1414" t="inlineStr">
+        <is>
+          <t>j123kcmcn</t>
+        </is>
+      </c>
+      <c r="H1414" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1414" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1414" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1414" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1414" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1415">
+      <c r="A1415" t="n">
+        <v>1414</v>
+      </c>
+      <c r="B1415" t="inlineStr">
+        <is>
+          <t>732223CC044</t>
+        </is>
+      </c>
+      <c r="C1415" t="inlineStr">
+        <is>
+          <t>RAM PRAKASH S</t>
+        </is>
+      </c>
+      <c r="D1415" t="inlineStr">
+        <is>
+          <t>CSE(CS)</t>
+        </is>
+      </c>
+      <c r="E1415" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="F1415" t="inlineStr">
+        <is>
+          <t>2023 - 2027</t>
+        </is>
+      </c>
+      <c r="G1415" t="inlineStr">
+        <is>
+          <t>raamprakash5</t>
+        </is>
+      </c>
+      <c r="H1415" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1415" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1415" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1415" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1415" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1416">
+      <c r="A1416" t="n">
+        <v>1415</v>
+      </c>
+      <c r="B1416" t="inlineStr">
+        <is>
+          <t>732223CC045</t>
+        </is>
+      </c>
+      <c r="C1416" t="inlineStr">
+        <is>
+          <t>RATHEESH S</t>
+        </is>
+      </c>
+      <c r="D1416" t="inlineStr">
+        <is>
+          <t>CSE(CS)</t>
+        </is>
+      </c>
+      <c r="E1416" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="F1416" t="inlineStr">
+        <is>
+          <t>2023 - 2027</t>
+        </is>
+      </c>
+      <c r="G1416" t="inlineStr">
+        <is>
+          <t>ratheesh1226</t>
+        </is>
+      </c>
+      <c r="H1416" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1416" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1416" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1416" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1416" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1417">
+      <c r="A1417" t="n">
+        <v>1416</v>
+      </c>
+      <c r="B1417" t="inlineStr">
+        <is>
+          <t>732223CC046</t>
+        </is>
+      </c>
+      <c r="C1417" t="inlineStr">
+        <is>
+          <t>RITHIKA P</t>
+        </is>
+      </c>
+      <c r="D1417" t="inlineStr">
+        <is>
+          <t>CSE(CS)</t>
+        </is>
+      </c>
+      <c r="E1417" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="F1417" t="inlineStr">
+        <is>
+          <t>2023 - 2027</t>
+        </is>
+      </c>
+      <c r="G1417" t="inlineStr">
+        <is>
+          <t>rithikapi13</t>
+        </is>
+      </c>
+      <c r="H1417" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1417" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1417" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1417" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1417" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1418">
+      <c r="A1418" t="n">
+        <v>1417</v>
+      </c>
+      <c r="B1418" t="inlineStr">
+        <is>
+          <t>732223CC047</t>
+        </is>
+      </c>
+      <c r="C1418" t="inlineStr">
+        <is>
+          <t>SARAVANAN R</t>
+        </is>
+      </c>
+      <c r="D1418" t="inlineStr">
+        <is>
+          <t>CSE(CS)</t>
+        </is>
+      </c>
+      <c r="E1418" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="F1418" t="inlineStr">
+        <is>
+          <t>2023 - 2027</t>
+        </is>
+      </c>
+      <c r="G1418" t="inlineStr">
+        <is>
+          <t>saravanan_rolex</t>
+        </is>
+      </c>
+      <c r="H1418" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1418" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1418" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1418" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1418" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1419">
+      <c r="A1419" t="n">
+        <v>1418</v>
+      </c>
+      <c r="B1419" t="inlineStr">
+        <is>
+          <t>732223CC050</t>
+        </is>
+      </c>
+      <c r="C1419" t="inlineStr">
+        <is>
+          <t>SRIVIDHYA S</t>
+        </is>
+      </c>
+      <c r="D1419" t="inlineStr">
+        <is>
+          <t>CSE(CS)</t>
+        </is>
+      </c>
+      <c r="E1419" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="F1419" t="inlineStr">
+        <is>
+          <t>2023 - 2027</t>
+        </is>
+      </c>
+      <c r="G1419" t="inlineStr">
+        <is>
+          <t>srividhya_25</t>
+        </is>
+      </c>
+      <c r="H1419" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1419" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1419" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1419" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1419" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1420">
+      <c r="A1420" t="n">
+        <v>1419</v>
+      </c>
+      <c r="B1420" t="inlineStr">
+        <is>
+          <t>732223CC051</t>
+        </is>
+      </c>
+      <c r="C1420" t="inlineStr">
+        <is>
+          <t>SRIRAM.S</t>
+        </is>
+      </c>
+      <c r="D1420" t="inlineStr">
+        <is>
+          <t>CSE(CS)</t>
+        </is>
+      </c>
+      <c r="E1420" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="F1420" t="inlineStr">
+        <is>
+          <t>2023 - 2027</t>
+        </is>
+      </c>
+      <c r="G1420" t="inlineStr">
+        <is>
+          <t>sriram6758</t>
+        </is>
+      </c>
+      <c r="H1420" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1420" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1420" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1420" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1420" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1421">
+      <c r="A1421" t="n">
+        <v>1420</v>
+      </c>
+      <c r="B1421" t="inlineStr">
+        <is>
+          <t>732223CC052</t>
+        </is>
+      </c>
+      <c r="C1421" t="inlineStr">
+        <is>
+          <t>STEFFY MARTINA P</t>
+        </is>
+      </c>
+      <c r="D1421" t="inlineStr">
+        <is>
+          <t>CSE(CS)</t>
+        </is>
+      </c>
+      <c r="E1421" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="F1421" t="inlineStr">
+        <is>
+          <t>2023 - 2027</t>
+        </is>
+      </c>
+      <c r="G1421" t="inlineStr">
+        <is>
+          <t>steffy_15</t>
+        </is>
+      </c>
+      <c r="H1421" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1421" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1421" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1421" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1421" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1422">
+      <c r="A1422" t="n">
+        <v>1421</v>
+      </c>
+      <c r="B1422" t="inlineStr">
+        <is>
+          <t>732223CC053</t>
+        </is>
+      </c>
+      <c r="C1422" t="inlineStr">
+        <is>
+          <t>SUBITHA P S</t>
+        </is>
+      </c>
+      <c r="D1422" t="inlineStr">
+        <is>
+          <t>CSE(CS)</t>
+        </is>
+      </c>
+      <c r="E1422" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="F1422" t="inlineStr">
+        <is>
+          <t>2023 - 2027</t>
+        </is>
+      </c>
+      <c r="G1422" t="inlineStr">
+        <is>
+          <t>23cc053</t>
+        </is>
+      </c>
+      <c r="H1422" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1422" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1422" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1422" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1422" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1423">
+      <c r="A1423" t="n">
+        <v>1422</v>
+      </c>
+      <c r="B1423" t="inlineStr">
+        <is>
+          <t>732223CC056</t>
+        </is>
+      </c>
+      <c r="C1423" t="inlineStr">
+        <is>
+          <t>VIGNESH J</t>
+        </is>
+      </c>
+      <c r="D1423" t="inlineStr">
+        <is>
+          <t>CSE(CS)</t>
+        </is>
+      </c>
+      <c r="E1423" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="F1423" t="inlineStr">
+        <is>
+          <t>2023 - 2027</t>
+        </is>
+      </c>
+      <c r="G1423" t="inlineStr">
+        <is>
+          <t>vignesh_2639</t>
+        </is>
+      </c>
+      <c r="H1423" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1423" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1423" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1423" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1423" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1424">
+      <c r="A1424" t="n">
+        <v>1423</v>
+      </c>
+      <c r="B1424" t="inlineStr">
+        <is>
+          <t>732223CC059</t>
+        </is>
+      </c>
+      <c r="C1424" t="inlineStr">
+        <is>
+          <t>WASIM M</t>
+        </is>
+      </c>
+      <c r="D1424" t="inlineStr">
+        <is>
+          <t>CSE(CS)</t>
+        </is>
+      </c>
+      <c r="E1424" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="F1424" t="inlineStr">
+        <is>
+          <t>2023 - 2027</t>
+        </is>
+      </c>
+      <c r="G1424" t="inlineStr">
+        <is>
+          <t>wasim_m</t>
+        </is>
+      </c>
+      <c r="H1424" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1424" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1424" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1424" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1424" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1425">
+      <c r="A1425" t="n">
+        <v>1424</v>
+      </c>
+      <c r="B1425" t="inlineStr">
+        <is>
+          <t>732223CI002</t>
+        </is>
+      </c>
+      <c r="C1425" t="inlineStr">
+        <is>
+          <t>AJAY VISHALESWAR</t>
+        </is>
+      </c>
+      <c r="D1425" t="inlineStr">
+        <is>
+          <t>CSE(IOT)</t>
+        </is>
+      </c>
+      <c r="E1425" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="F1425" t="inlineStr">
+        <is>
+          <t>2023 - 2027</t>
+        </is>
+      </c>
+      <c r="G1425" t="inlineStr">
+        <is>
+          <t>ajaysoftware</t>
+        </is>
+      </c>
+      <c r="H1425" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1425" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1425" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1425" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1425" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1426">
+      <c r="A1426" t="n">
+        <v>1425</v>
+      </c>
+      <c r="B1426" t="inlineStr">
+        <is>
+          <t>732223CI004</t>
+        </is>
+      </c>
+      <c r="C1426" t="inlineStr">
+        <is>
+          <t>BHUVANADHARSHINI C</t>
+        </is>
+      </c>
+      <c r="D1426" t="inlineStr">
+        <is>
+          <t>CSE(IOT)</t>
+        </is>
+      </c>
+      <c r="E1426" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="F1426" t="inlineStr">
+        <is>
+          <t>2023 - 2027</t>
+        </is>
+      </c>
+      <c r="G1426" t="inlineStr">
+        <is>
+          <t>bhuvanadharshini</t>
+        </is>
+      </c>
+      <c r="H1426" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1426" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1426" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1426" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1426" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1427">
+      <c r="A1427" t="n">
+        <v>1426</v>
+      </c>
+      <c r="B1427" t="inlineStr">
+        <is>
+          <t>732223CI006</t>
+        </is>
+      </c>
+      <c r="C1427" t="inlineStr">
+        <is>
+          <t>DHARNEESH P</t>
+        </is>
+      </c>
+      <c r="D1427" t="inlineStr">
+        <is>
+          <t>CSE(IOT)</t>
+        </is>
+      </c>
+      <c r="E1427" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="F1427" t="inlineStr">
+        <is>
+          <t>2023 - 2027</t>
+        </is>
+      </c>
+      <c r="G1427" t="inlineStr">
+        <is>
+          <t>tdq3hurfei</t>
+        </is>
+      </c>
+      <c r="H1427" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1427" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1427" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1427" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1427" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1428">
+      <c r="A1428" t="n">
+        <v>1427</v>
+      </c>
+      <c r="B1428" t="inlineStr">
+        <is>
+          <t>732223CI007</t>
+        </is>
+      </c>
+      <c r="C1428" t="inlineStr">
+        <is>
+          <t>DIVYA A</t>
+        </is>
+      </c>
+      <c r="D1428" t="inlineStr">
+        <is>
+          <t>CSE(IOT)</t>
+        </is>
+      </c>
+      <c r="E1428" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="F1428" t="inlineStr">
+        <is>
+          <t>2023 - 2027</t>
+        </is>
+      </c>
+      <c r="G1428" t="inlineStr">
+        <is>
+          <t>DIVI_ARUL</t>
+        </is>
+      </c>
+      <c r="H1428" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1428" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1428" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1428" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1428" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1429">
+      <c r="A1429" t="n">
+        <v>1428</v>
+      </c>
+      <c r="B1429" t="inlineStr">
+        <is>
+          <t>732223CI010</t>
+        </is>
+      </c>
+      <c r="C1429" t="inlineStr">
+        <is>
+          <t>GOKILA.G</t>
+        </is>
+      </c>
+      <c r="D1429" t="inlineStr">
+        <is>
+          <t>CSE(IOT)</t>
+        </is>
+      </c>
+      <c r="E1429" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="F1429" t="inlineStr">
+        <is>
+          <t>2023 - 2027</t>
+        </is>
+      </c>
+      <c r="G1429" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H1429" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1429" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1429" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1429" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1429" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1430">
+      <c r="A1430" t="n">
+        <v>1429</v>
+      </c>
+      <c r="B1430" t="inlineStr">
+        <is>
+          <t>732223CI012</t>
+        </is>
+      </c>
+      <c r="C1430" t="inlineStr">
+        <is>
+          <t>GOWCIKA U</t>
+        </is>
+      </c>
+      <c r="D1430" t="inlineStr">
+        <is>
+          <t>CSE(IOT)</t>
+        </is>
+      </c>
+      <c r="E1430" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="F1430" t="inlineStr">
+        <is>
+          <t>2023 - 2027</t>
+        </is>
+      </c>
+      <c r="G1430" t="inlineStr">
+        <is>
+          <t>Gowcika</t>
+        </is>
+      </c>
+      <c r="H1430" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1430" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1430" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1430" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1430" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1431">
+      <c r="A1431" t="n">
+        <v>1430</v>
+      </c>
+      <c r="B1431" t="inlineStr">
+        <is>
+          <t>732223CI013</t>
+        </is>
+      </c>
+      <c r="C1431" t="inlineStr">
+        <is>
+          <t>HAMSHA N</t>
+        </is>
+      </c>
+      <c r="D1431" t="inlineStr">
+        <is>
+          <t>CSE(IOT)</t>
+        </is>
+      </c>
+      <c r="E1431" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="F1431" t="inlineStr">
+        <is>
+          <t>2023 - 2027</t>
+        </is>
+      </c>
+      <c r="G1431" t="inlineStr">
+        <is>
+          <t>hamsha07</t>
+        </is>
+      </c>
+      <c r="H1431" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1431" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1431" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1431" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1431" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1432">
+      <c r="A1432" t="n">
+        <v>1431</v>
+      </c>
+      <c r="B1432" t="inlineStr">
+        <is>
+          <t>732223CI014</t>
+        </is>
+      </c>
+      <c r="C1432" t="inlineStr">
+        <is>
+          <t>HAREE D</t>
+        </is>
+      </c>
+      <c r="D1432" t="inlineStr">
+        <is>
+          <t>CSE(IOT)</t>
+        </is>
+      </c>
+      <c r="E1432" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="F1432" t="inlineStr">
+        <is>
+          <t>2023 - 2027</t>
+        </is>
+      </c>
+      <c r="G1432" t="inlineStr">
+        <is>
+          <t>Haree05</t>
+        </is>
+      </c>
+      <c r="H1432" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1432" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1432" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1432" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1432" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1433">
+      <c r="A1433" t="n">
+        <v>1432</v>
+      </c>
+      <c r="B1433" t="inlineStr">
+        <is>
+          <t>732223CI015</t>
+        </is>
+      </c>
+      <c r="C1433" t="inlineStr">
+        <is>
+          <t>HARINI S</t>
+        </is>
+      </c>
+      <c r="D1433" t="inlineStr">
+        <is>
+          <t>CSE(IOT)</t>
+        </is>
+      </c>
+      <c r="E1433" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="F1433" t="inlineStr">
+        <is>
+          <t>2023 - 2027</t>
+        </is>
+      </c>
+      <c r="G1433" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H1433" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1433" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1433" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1433" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1433" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1434">
+      <c r="A1434" t="n">
+        <v>1433</v>
+      </c>
+      <c r="B1434" t="inlineStr">
+        <is>
+          <t>732223CI018</t>
+        </is>
+      </c>
+      <c r="C1434" t="inlineStr">
+        <is>
+          <t>JAYASURYA P</t>
+        </is>
+      </c>
+      <c r="D1434" t="inlineStr">
+        <is>
+          <t>CSE(IOT)</t>
+        </is>
+      </c>
+      <c r="E1434" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="F1434" t="inlineStr">
+        <is>
+          <t>2023 - 2027</t>
+        </is>
+      </c>
+      <c r="G1434" t="inlineStr">
+        <is>
+          <t>Jayasurya-619</t>
+        </is>
+      </c>
+      <c r="H1434" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1434" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1434" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1434" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1434" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1435">
+      <c r="A1435" t="n">
+        <v>1434</v>
+      </c>
+      <c r="B1435" t="inlineStr">
+        <is>
+          <t>732223CI021</t>
+        </is>
+      </c>
+      <c r="C1435" t="inlineStr">
+        <is>
+          <t>KAMALA VISHNU G</t>
+        </is>
+      </c>
+      <c r="D1435" t="inlineStr">
+        <is>
+          <t>CSE(IOT)</t>
+        </is>
+      </c>
+      <c r="E1435" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="F1435" t="inlineStr">
+        <is>
+          <t>2023 - 2027</t>
+        </is>
+      </c>
+      <c r="G1435" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H1435" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1435" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1435" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1435" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1435" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1436">
+      <c r="A1436" t="n">
+        <v>1435</v>
+      </c>
+      <c r="B1436" t="inlineStr">
+        <is>
+          <t>732223CI022</t>
+        </is>
+      </c>
+      <c r="C1436" t="inlineStr">
+        <is>
+          <t>KARMUKILAN A</t>
+        </is>
+      </c>
+      <c r="D1436" t="inlineStr">
+        <is>
+          <t>CSE(IOT)</t>
+        </is>
+      </c>
+      <c r="E1436" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="F1436" t="inlineStr">
+        <is>
+          <t>2023 - 2027</t>
+        </is>
+      </c>
+      <c r="G1436" t="inlineStr">
+        <is>
+          <t>pPPRNale4T</t>
+        </is>
+      </c>
+      <c r="H1436" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1436" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1436" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1436" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1436" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1437">
+      <c r="A1437" t="n">
+        <v>1436</v>
+      </c>
+      <c r="B1437" t="inlineStr">
+        <is>
+          <t>732223CI023</t>
+        </is>
+      </c>
+      <c r="C1437" t="inlineStr">
+        <is>
+          <t>KARTHIK.V</t>
+        </is>
+      </c>
+      <c r="D1437" t="inlineStr">
+        <is>
+          <t>CSE(IOT)</t>
+        </is>
+      </c>
+      <c r="E1437" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="F1437" t="inlineStr">
+        <is>
+          <t>2023 - 2027</t>
+        </is>
+      </c>
+      <c r="G1437" t="inlineStr">
+        <is>
+          <t>karthik_v3</t>
+        </is>
+      </c>
+      <c r="H1437" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1437" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1437" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1437" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1437" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1438">
+      <c r="A1438" t="n">
+        <v>1437</v>
+      </c>
+      <c r="B1438" t="inlineStr">
+        <is>
+          <t>732223CI025</t>
+        </is>
+      </c>
+      <c r="C1438" t="inlineStr">
+        <is>
+          <t>KARUNYA C</t>
+        </is>
+      </c>
+      <c r="D1438" t="inlineStr">
+        <is>
+          <t>CSE(IOT)</t>
+        </is>
+      </c>
+      <c r="E1438" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="F1438" t="inlineStr">
+        <is>
+          <t>2023 - 2027</t>
+        </is>
+      </c>
+      <c r="G1438" t="inlineStr">
+        <is>
+          <t>sivakarunya</t>
+        </is>
+      </c>
+      <c r="H1438" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1438" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1438" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1438" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1438" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1439">
+      <c r="A1439" t="n">
+        <v>1438</v>
+      </c>
+      <c r="B1439" t="inlineStr">
+        <is>
+          <t>732223CI027</t>
+        </is>
+      </c>
+      <c r="C1439" t="inlineStr">
+        <is>
+          <t>KAVI ISHWARRYA S K</t>
+        </is>
+      </c>
+      <c r="D1439" t="inlineStr">
+        <is>
+          <t>CSE(IOT)</t>
+        </is>
+      </c>
+      <c r="E1439" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="F1439" t="inlineStr">
+        <is>
+          <t>2023 - 2027</t>
+        </is>
+      </c>
+      <c r="G1439" t="inlineStr">
+        <is>
+          <t>s9hXtuAA2E</t>
+        </is>
+      </c>
+      <c r="H1439" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1439" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1439" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1439" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1439" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1440">
+      <c r="A1440" t="n">
+        <v>1439</v>
+      </c>
+      <c r="B1440" t="inlineStr">
+        <is>
+          <t>732223CI028</t>
+        </is>
+      </c>
+      <c r="C1440" t="inlineStr">
+        <is>
+          <t>KAVIN V</t>
+        </is>
+      </c>
+      <c r="D1440" t="inlineStr">
+        <is>
+          <t>CSE(IOT)</t>
+        </is>
+      </c>
+      <c r="E1440" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="F1440" t="inlineStr">
+        <is>
+          <t>2023 - 2027</t>
+        </is>
+      </c>
+      <c r="G1440" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H1440" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1440" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1440" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1440" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1440" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1441">
+      <c r="A1441" t="n">
+        <v>1440</v>
+      </c>
+      <c r="B1441" t="inlineStr">
+        <is>
+          <t>732223CI029</t>
+        </is>
+      </c>
+      <c r="C1441" t="inlineStr">
+        <is>
+          <t>KAVIYARASU S</t>
+        </is>
+      </c>
+      <c r="D1441" t="inlineStr">
+        <is>
+          <t>CSE(IOT)</t>
+        </is>
+      </c>
+      <c r="E1441" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="F1441" t="inlineStr">
+        <is>
+          <t>2023 - 2027</t>
+        </is>
+      </c>
+      <c r="G1441" t="inlineStr">
+        <is>
+          <t>KAVIYARASU_S123</t>
+        </is>
+      </c>
+      <c r="H1441" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1441" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1441" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1441" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1441" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1442">
+      <c r="A1442" t="n">
+        <v>1441</v>
+      </c>
+      <c r="B1442" t="inlineStr">
+        <is>
+          <t>732223CI030</t>
+        </is>
+      </c>
+      <c r="C1442" t="inlineStr">
+        <is>
+          <t>KEERTHANA K</t>
+        </is>
+      </c>
+      <c r="D1442" t="inlineStr">
+        <is>
+          <t>CSE(IOT)</t>
+        </is>
+      </c>
+      <c r="E1442" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="F1442" t="inlineStr">
+        <is>
+          <t>2023 - 2027</t>
+        </is>
+      </c>
+      <c r="G1442" t="inlineStr">
+        <is>
+          <t>K_KEERTHANA_</t>
+        </is>
+      </c>
+      <c r="H1442" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1442" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1442" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1442" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1442" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1443">
+      <c r="A1443" t="n">
+        <v>1442</v>
+      </c>
+      <c r="B1443" t="inlineStr">
+        <is>
+          <t>732223CI034</t>
+        </is>
+      </c>
+      <c r="C1443" t="inlineStr">
+        <is>
+          <t>MOHAMED AQDHAS U</t>
+        </is>
+      </c>
+      <c r="D1443" t="inlineStr">
+        <is>
+          <t>CSE(IOT)</t>
+        </is>
+      </c>
+      <c r="E1443" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="F1443" t="inlineStr">
+        <is>
+          <t>2023 - 2027</t>
+        </is>
+      </c>
+      <c r="G1443" t="inlineStr">
+        <is>
+          <t>AQDHAS</t>
+        </is>
+      </c>
+      <c r="H1443" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1443" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1443" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1443" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1443" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1444">
+      <c r="A1444" t="n">
+        <v>1443</v>
+      </c>
+      <c r="B1444" t="inlineStr">
+        <is>
+          <t>732223CI038</t>
+        </is>
+      </c>
+      <c r="C1444" t="inlineStr">
+        <is>
+          <t>PRABHAKARAN . S</t>
+        </is>
+      </c>
+      <c r="D1444" t="inlineStr">
+        <is>
+          <t>CSE(IOT)</t>
+        </is>
+      </c>
+      <c r="E1444" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="F1444" t="inlineStr">
+        <is>
+          <t>2023 - 2027</t>
+        </is>
+      </c>
+      <c r="G1444" t="inlineStr">
+        <is>
+          <t>Prabha_1503</t>
+        </is>
+      </c>
+      <c r="H1444" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1444" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1444" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1444" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1444" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1445">
+      <c r="A1445" t="n">
+        <v>1444</v>
+      </c>
+      <c r="B1445" t="inlineStr">
+        <is>
+          <t>732223CI044</t>
+        </is>
+      </c>
+      <c r="C1445" t="inlineStr">
+        <is>
+          <t>RAVI BHARATHI.J</t>
+        </is>
+      </c>
+      <c r="D1445" t="inlineStr">
+        <is>
+          <t>CSE(IOT)</t>
+        </is>
+      </c>
+      <c r="E1445" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="F1445" t="inlineStr">
+        <is>
+          <t>2023 - 2027</t>
+        </is>
+      </c>
+      <c r="G1445" t="inlineStr">
+        <is>
+          <t>ravi_bharathi509</t>
+        </is>
+      </c>
+      <c r="H1445" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1445" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1445" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1445" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1445" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1446">
+      <c r="A1446" t="n">
+        <v>1445</v>
+      </c>
+      <c r="B1446" t="inlineStr">
+        <is>
+          <t>732223CI046</t>
+        </is>
+      </c>
+      <c r="C1446" t="inlineStr">
+        <is>
+          <t>ROHITH T</t>
+        </is>
+      </c>
+      <c r="D1446" t="inlineStr">
+        <is>
+          <t>CSE(IOT)</t>
+        </is>
+      </c>
+      <c r="E1446" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="F1446" t="inlineStr">
+        <is>
+          <t>2023 - 2027</t>
+        </is>
+      </c>
+      <c r="G1446" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H1446" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1446" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1446" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1446" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1446" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1447">
+      <c r="A1447" t="n">
+        <v>1446</v>
+      </c>
+      <c r="B1447" t="inlineStr">
+        <is>
+          <t>732223CI050</t>
+        </is>
+      </c>
+      <c r="C1447" t="inlineStr">
+        <is>
+          <t>SATHISHKUMAR.S</t>
+        </is>
+      </c>
+      <c r="D1447" t="inlineStr">
+        <is>
+          <t>CSE(IOT)</t>
+        </is>
+      </c>
+      <c r="E1447" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="F1447" t="inlineStr">
+        <is>
+          <t>2023 - 2027</t>
+        </is>
+      </c>
+      <c r="G1447" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H1447" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1447" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1447" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1447" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1447" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1448">
+      <c r="A1448" t="n">
+        <v>1447</v>
+      </c>
+      <c r="B1448" t="inlineStr">
+        <is>
+          <t>732223CI053</t>
+        </is>
+      </c>
+      <c r="C1448" t="inlineStr">
+        <is>
+          <t>SUJITH K</t>
+        </is>
+      </c>
+      <c r="D1448" t="inlineStr">
+        <is>
+          <t>CSE(IOT)</t>
+        </is>
+      </c>
+      <c r="E1448" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="F1448" t="inlineStr">
+        <is>
+          <t>2023 - 2027</t>
+        </is>
+      </c>
+      <c r="G1448" t="inlineStr">
+        <is>
+          <t>sujith2006</t>
+        </is>
+      </c>
+      <c r="H1448" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1448" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1448" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1448" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1448" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1449">
+      <c r="A1449" t="n">
+        <v>1448</v>
+      </c>
+      <c r="B1449" t="inlineStr">
+        <is>
+          <t>732223CI055</t>
+        </is>
+      </c>
+      <c r="C1449" t="inlineStr">
+        <is>
+          <t>G THEJASWINI</t>
+        </is>
+      </c>
+      <c r="D1449" t="inlineStr">
+        <is>
+          <t>CSE(IOT)</t>
+        </is>
+      </c>
+      <c r="E1449" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="F1449" t="inlineStr">
+        <is>
+          <t>2023 - 2027</t>
+        </is>
+      </c>
+      <c r="G1449" t="inlineStr">
+        <is>
+          <t>thejaswini_10</t>
+        </is>
+      </c>
+      <c r="H1449" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1449" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1449" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1449" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1449" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1450">
+      <c r="A1450" t="n">
+        <v>1449</v>
+      </c>
+      <c r="B1450" t="inlineStr">
+        <is>
+          <t>732223CI058</t>
+        </is>
+      </c>
+      <c r="C1450" t="inlineStr">
+        <is>
+          <t>VICHITHRA.V</t>
+        </is>
+      </c>
+      <c r="D1450" t="inlineStr">
+        <is>
+          <t>CSE(IOT)</t>
+        </is>
+      </c>
+      <c r="E1450" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="F1450" t="inlineStr">
+        <is>
+          <t>2023 - 2027</t>
+        </is>
+      </c>
+      <c r="G1450" t="inlineStr">
+        <is>
+          <t>VichithraVelusamy</t>
+        </is>
+      </c>
+      <c r="H1450" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1450" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1450" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1450" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1450" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1451">
+      <c r="A1451" t="n">
+        <v>1450</v>
+      </c>
+      <c r="B1451" t="inlineStr">
+        <is>
+          <t>732223CI001</t>
+        </is>
+      </c>
+      <c r="C1451" t="inlineStr">
+        <is>
+          <t>AAKASH SHIVA KB</t>
+        </is>
+      </c>
+      <c r="D1451" t="inlineStr">
+        <is>
+          <t>CSE(IOT)</t>
+        </is>
+      </c>
+      <c r="E1451" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="F1451" t="inlineStr">
+        <is>
+          <t>2023 - 2027</t>
+        </is>
+      </c>
+      <c r="G1451" t="inlineStr">
+        <is>
+          <t>aakashshiva</t>
+        </is>
+      </c>
+      <c r="H1451" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1451" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1451" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1451" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1451" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1452">
+      <c r="A1452" t="n">
+        <v>1451</v>
+      </c>
+      <c r="B1452" t="inlineStr">
+        <is>
+          <t>732223CS01451</t>
+        </is>
+      </c>
+      <c r="C1452" t="inlineStr">
+        <is>
+          <t>Student 01451 (CS)</t>
+        </is>
+      </c>
+      <c r="D1452" t="inlineStr">
+        <is>
+          <t>CSE(CS)</t>
+        </is>
+      </c>
+      <c r="E1452" t="inlineStr">
+        <is>
+          <t>III</t>
+        </is>
+      </c>
+      <c r="F1452" t="inlineStr">
+        <is>
+          <t>2024 - 2028</t>
+        </is>
+      </c>
+      <c r="G1452" t="inlineStr">
+        <is>
+          <t>coder_cs_1451</t>
+        </is>
+      </c>
+      <c r="H1452" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1452" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1452" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1452" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1452" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1453">
+      <c r="A1453" t="n">
+        <v>1452</v>
+      </c>
+      <c r="B1453" t="inlineStr">
+        <is>
+          <t>732223CS01452</t>
+        </is>
+      </c>
+      <c r="C1453" t="inlineStr">
+        <is>
+          <t>Student 01452 (CS)</t>
+        </is>
+      </c>
+      <c r="D1453" t="inlineStr">
+        <is>
+          <t>CSE(CS)</t>
+        </is>
+      </c>
+      <c r="E1453" t="inlineStr">
+        <is>
+          <t>III</t>
+        </is>
+      </c>
+      <c r="F1453" t="inlineStr">
+        <is>
+          <t>2024 - 2028</t>
+        </is>
+      </c>
+      <c r="G1453" t="inlineStr">
+        <is>
+          <t>coder_cs_1452</t>
+        </is>
+      </c>
+      <c r="H1453" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1453" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1453" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1453" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1453" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1454">
+      <c r="A1454" t="n">
+        <v>1453</v>
+      </c>
+      <c r="B1454" t="inlineStr">
+        <is>
+          <t>732223CS01453</t>
+        </is>
+      </c>
+      <c r="C1454" t="inlineStr">
+        <is>
+          <t>Student 01453 (CS)</t>
+        </is>
+      </c>
+      <c r="D1454" t="inlineStr">
+        <is>
+          <t>CSE(CS)</t>
+        </is>
+      </c>
+      <c r="E1454" t="inlineStr">
+        <is>
+          <t>III</t>
+        </is>
+      </c>
+      <c r="F1454" t="inlineStr">
+        <is>
+          <t>2024 - 2028</t>
+        </is>
+      </c>
+      <c r="G1454" t="inlineStr">
+        <is>
+          <t>coder_cs_1453</t>
+        </is>
+      </c>
+      <c r="H1454" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1454" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1454" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1454" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1454" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1455">
+      <c r="A1455" t="n">
+        <v>1454</v>
+      </c>
+      <c r="B1455" t="inlineStr">
+        <is>
+          <t>732223CS01454</t>
+        </is>
+      </c>
+      <c r="C1455" t="inlineStr">
+        <is>
+          <t>Student 01454 (CS)</t>
+        </is>
+      </c>
+      <c r="D1455" t="inlineStr">
+        <is>
+          <t>CSE(CS)</t>
+        </is>
+      </c>
+      <c r="E1455" t="inlineStr">
+        <is>
+          <t>III</t>
+        </is>
+      </c>
+      <c r="F1455" t="inlineStr">
+        <is>
+          <t>2024 - 2028</t>
+        </is>
+      </c>
+      <c r="G1455" t="inlineStr">
+        <is>
+          <t>coder_cs_1454</t>
+        </is>
+      </c>
+      <c r="H1455" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1455" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1455" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1455" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1455" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1456">
+      <c r="A1456" t="n">
+        <v>1455</v>
+      </c>
+      <c r="B1456" t="inlineStr">
+        <is>
+          <t>732223CS01455</t>
+        </is>
+      </c>
+      <c r="C1456" t="inlineStr">
+        <is>
+          <t>Student 01455 (CS)</t>
+        </is>
+      </c>
+      <c r="D1456" t="inlineStr">
+        <is>
+          <t>CSE(CS)</t>
+        </is>
+      </c>
+      <c r="E1456" t="inlineStr">
+        <is>
+          <t>III</t>
+        </is>
+      </c>
+      <c r="F1456" t="inlineStr">
+        <is>
+          <t>2024 - 2028</t>
+        </is>
+      </c>
+      <c r="G1456" t="inlineStr">
+        <is>
+          <t>coder_cs_1455</t>
+        </is>
+      </c>
+      <c r="H1456" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1456" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1456" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1456" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1456" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1457">
+      <c r="A1457" t="n">
+        <v>1456</v>
+      </c>
+      <c r="B1457" t="inlineStr">
+        <is>
+          <t>732223CS01456</t>
+        </is>
+      </c>
+      <c r="C1457" t="inlineStr">
+        <is>
+          <t>Student 01456 (CS)</t>
+        </is>
+      </c>
+      <c r="D1457" t="inlineStr">
+        <is>
+          <t>CSE(CS)</t>
+        </is>
+      </c>
+      <c r="E1457" t="inlineStr">
+        <is>
+          <t>III</t>
+        </is>
+      </c>
+      <c r="F1457" t="inlineStr">
+        <is>
+          <t>2024 - 2028</t>
+        </is>
+      </c>
+      <c r="G1457" t="inlineStr">
+        <is>
+          <t>coder_cs_1456</t>
+        </is>
+      </c>
+      <c r="H1457" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1457" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1457" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1457" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1457" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1458">
+      <c r="A1458" t="n">
+        <v>1457</v>
+      </c>
+      <c r="B1458" t="inlineStr">
+        <is>
+          <t>732223CS01457</t>
+        </is>
+      </c>
+      <c r="C1458" t="inlineStr">
+        <is>
+          <t>Student 01457 (CS)</t>
+        </is>
+      </c>
+      <c r="D1458" t="inlineStr">
+        <is>
+          <t>CSE(CS)</t>
+        </is>
+      </c>
+      <c r="E1458" t="inlineStr">
+        <is>
+          <t>III</t>
+        </is>
+      </c>
+      <c r="F1458" t="inlineStr">
+        <is>
+          <t>2024 - 2028</t>
+        </is>
+      </c>
+      <c r="G1458" t="inlineStr">
+        <is>
+          <t>coder_cs_1457</t>
+        </is>
+      </c>
+      <c r="H1458" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1458" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1458" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1458" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1458" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1459">
+      <c r="A1459" t="n">
+        <v>1458</v>
+      </c>
+      <c r="B1459" t="inlineStr">
+        <is>
+          <t>732223CS01458</t>
+        </is>
+      </c>
+      <c r="C1459" t="inlineStr">
+        <is>
+          <t>Student 01458 (CS)</t>
+        </is>
+      </c>
+      <c r="D1459" t="inlineStr">
+        <is>
+          <t>CSE(CS)</t>
+        </is>
+      </c>
+      <c r="E1459" t="inlineStr">
+        <is>
+          <t>III</t>
+        </is>
+      </c>
+      <c r="F1459" t="inlineStr">
+        <is>
+          <t>2024 - 2028</t>
+        </is>
+      </c>
+      <c r="G1459" t="inlineStr">
+        <is>
+          <t>coder_cs_1458</t>
+        </is>
+      </c>
+      <c r="H1459" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1459" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1459" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1459" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1459" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1460">
+      <c r="A1460" t="n">
+        <v>1459</v>
+      </c>
+      <c r="B1460" t="inlineStr">
+        <is>
+          <t>732223CS01459</t>
+        </is>
+      </c>
+      <c r="C1460" t="inlineStr">
+        <is>
+          <t>Student 01459 (CS)</t>
+        </is>
+      </c>
+      <c r="D1460" t="inlineStr">
+        <is>
+          <t>CSE(CS)</t>
+        </is>
+      </c>
+      <c r="E1460" t="inlineStr">
+        <is>
+          <t>III</t>
+        </is>
+      </c>
+      <c r="F1460" t="inlineStr">
+        <is>
+          <t>2024 - 2028</t>
+        </is>
+      </c>
+      <c r="G1460" t="inlineStr">
+        <is>
+          <t>coder_cs_1459</t>
+        </is>
+      </c>
+      <c r="H1460" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1460" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1460" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1460" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1460" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1461">
+      <c r="A1461" t="n">
+        <v>1460</v>
+      </c>
+      <c r="B1461" t="inlineStr">
+        <is>
+          <t>732223CS01460</t>
+        </is>
+      </c>
+      <c r="C1461" t="inlineStr">
+        <is>
+          <t>Student 01460 (CS)</t>
+        </is>
+      </c>
+      <c r="D1461" t="inlineStr">
+        <is>
+          <t>CSE(CS)</t>
+        </is>
+      </c>
+      <c r="E1461" t="inlineStr">
+        <is>
+          <t>III</t>
+        </is>
+      </c>
+      <c r="F1461" t="inlineStr">
+        <is>
+          <t>2024 - 2028</t>
+        </is>
+      </c>
+      <c r="G1461" t="inlineStr">
+        <is>
+          <t>coder_cs_1460</t>
+        </is>
+      </c>
+      <c r="H1461" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1461" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1461" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1461" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1461" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1462">
+      <c r="A1462" t="n">
+        <v>1461</v>
+      </c>
+      <c r="B1462" t="inlineStr">
+        <is>
+          <t>732223CS01461</t>
+        </is>
+      </c>
+      <c r="C1462" t="inlineStr">
+        <is>
+          <t>Student 01461 (CS)</t>
+        </is>
+      </c>
+      <c r="D1462" t="inlineStr">
+        <is>
+          <t>CSE(CS)</t>
+        </is>
+      </c>
+      <c r="E1462" t="inlineStr">
+        <is>
+          <t>III</t>
+        </is>
+      </c>
+      <c r="F1462" t="inlineStr">
+        <is>
+          <t>2024 - 2028</t>
+        </is>
+      </c>
+      <c r="G1462" t="inlineStr">
+        <is>
+          <t>coder_cs_1461</t>
+        </is>
+      </c>
+      <c r="H1462" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1462" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1462" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1462" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1462" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1463">
+      <c r="A1463" t="n">
+        <v>1462</v>
+      </c>
+      <c r="B1463" t="inlineStr">
+        <is>
+          <t>732223CS01462</t>
+        </is>
+      </c>
+      <c r="C1463" t="inlineStr">
+        <is>
+          <t>Student 01462 (CS)</t>
+        </is>
+      </c>
+      <c r="D1463" t="inlineStr">
+        <is>
+          <t>CSE(CS)</t>
+        </is>
+      </c>
+      <c r="E1463" t="inlineStr">
+        <is>
+          <t>III</t>
+        </is>
+      </c>
+      <c r="F1463" t="inlineStr">
+        <is>
+          <t>2024 - 2028</t>
+        </is>
+      </c>
+      <c r="G1463" t="inlineStr">
+        <is>
+          <t>coder_cs_1462</t>
+        </is>
+      </c>
+      <c r="H1463" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1463" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1463" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1463" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1463" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1464">
+      <c r="A1464" t="n">
+        <v>1463</v>
+      </c>
+      <c r="B1464" t="inlineStr">
+        <is>
+          <t>732223CS01463</t>
+        </is>
+      </c>
+      <c r="C1464" t="inlineStr">
+        <is>
+          <t>Student 01463 (CS)</t>
+        </is>
+      </c>
+      <c r="D1464" t="inlineStr">
+        <is>
+          <t>CSE(CS)</t>
+        </is>
+      </c>
+      <c r="E1464" t="inlineStr">
+        <is>
+          <t>III</t>
+        </is>
+      </c>
+      <c r="F1464" t="inlineStr">
+        <is>
+          <t>2024 - 2028</t>
+        </is>
+      </c>
+      <c r="G1464" t="inlineStr">
+        <is>
+          <t>coder_cs_1463</t>
+        </is>
+      </c>
+      <c r="H1464" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1464" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1464" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1464" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1464" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1465">
+      <c r="A1465" t="n">
+        <v>1464</v>
+      </c>
+      <c r="B1465" t="inlineStr">
+        <is>
+          <t>732223CS01464</t>
+        </is>
+      </c>
+      <c r="C1465" t="inlineStr">
+        <is>
+          <t>Student 01464 (CS)</t>
+        </is>
+      </c>
+      <c r="D1465" t="inlineStr">
+        <is>
+          <t>CSE(CS)</t>
+        </is>
+      </c>
+      <c r="E1465" t="inlineStr">
+        <is>
+          <t>III</t>
+        </is>
+      </c>
+      <c r="F1465" t="inlineStr">
+        <is>
+          <t>2024 - 2028</t>
+        </is>
+      </c>
+      <c r="G1465" t="inlineStr">
+        <is>
+          <t>coder_cs_1464</t>
+        </is>
+      </c>
+      <c r="H1465" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1465" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1465" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1465" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1465" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1466">
+      <c r="A1466" t="n">
+        <v>1465</v>
+      </c>
+      <c r="B1466" t="inlineStr">
+        <is>
+          <t>732223CS01465</t>
+        </is>
+      </c>
+      <c r="C1466" t="inlineStr">
+        <is>
+          <t>Student 01465 (CS)</t>
+        </is>
+      </c>
+      <c r="D1466" t="inlineStr">
+        <is>
+          <t>CSE(CS)</t>
+        </is>
+      </c>
+      <c r="E1466" t="inlineStr">
+        <is>
+          <t>III</t>
+        </is>
+      </c>
+      <c r="F1466" t="inlineStr">
+        <is>
+          <t>2024 - 2028</t>
+        </is>
+      </c>
+      <c r="G1466" t="inlineStr">
+        <is>
+          <t>coder_cs_1465</t>
+        </is>
+      </c>
+      <c r="H1466" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1466" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1466" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1466" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1466" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1467">
+      <c r="A1467" t="n">
+        <v>1466</v>
+      </c>
+      <c r="B1467" t="inlineStr">
+        <is>
+          <t>732223CS01466</t>
+        </is>
+      </c>
+      <c r="C1467" t="inlineStr">
+        <is>
+          <t>Student 01466 (CS)</t>
+        </is>
+      </c>
+      <c r="D1467" t="inlineStr">
+        <is>
+          <t>CSE(CS)</t>
+        </is>
+      </c>
+      <c r="E1467" t="inlineStr">
+        <is>
+          <t>III</t>
+        </is>
+      </c>
+      <c r="F1467" t="inlineStr">
+        <is>
+          <t>2024 - 2028</t>
+        </is>
+      </c>
+      <c r="G1467" t="inlineStr">
+        <is>
+          <t>coder_cs_1466</t>
+        </is>
+      </c>
+      <c r="H1467" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1467" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1467" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1467" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1467" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1468">
+      <c r="A1468" t="n">
+        <v>1467</v>
+      </c>
+      <c r="B1468" t="inlineStr">
+        <is>
+          <t>732223CS01467</t>
+        </is>
+      </c>
+      <c r="C1468" t="inlineStr">
+        <is>
+          <t>Student 01467 (CS)</t>
+        </is>
+      </c>
+      <c r="D1468" t="inlineStr">
+        <is>
+          <t>CSE(CS)</t>
+        </is>
+      </c>
+      <c r="E1468" t="inlineStr">
+        <is>
+          <t>III</t>
+        </is>
+      </c>
+      <c r="F1468" t="inlineStr">
+        <is>
+          <t>2024 - 2028</t>
+        </is>
+      </c>
+      <c r="G1468" t="inlineStr">
+        <is>
+          <t>coder_cs_1467</t>
+        </is>
+      </c>
+      <c r="H1468" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1468" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1468" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1468" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1468" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1469">
+      <c r="A1469" t="n">
+        <v>1468</v>
+      </c>
+      <c r="B1469" t="inlineStr">
+        <is>
+          <t>732223CS01468</t>
+        </is>
+      </c>
+      <c r="C1469" t="inlineStr">
+        <is>
+          <t>Student 01468 (CS)</t>
+        </is>
+      </c>
+      <c r="D1469" t="inlineStr">
+        <is>
+          <t>CSE(CS)</t>
+        </is>
+      </c>
+      <c r="E1469" t="inlineStr">
+        <is>
+          <t>III</t>
+        </is>
+      </c>
+      <c r="F1469" t="inlineStr">
+        <is>
+          <t>2024 - 2028</t>
+        </is>
+      </c>
+      <c r="G1469" t="inlineStr">
+        <is>
+          <t>coder_cs_1468</t>
+        </is>
+      </c>
+      <c r="H1469" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1469" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1469" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1469" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1469" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1470">
+      <c r="A1470" t="n">
+        <v>1469</v>
+      </c>
+      <c r="B1470" t="inlineStr">
+        <is>
+          <t>732223CS01469</t>
+        </is>
+      </c>
+      <c r="C1470" t="inlineStr">
+        <is>
+          <t>Student 01469 (CS)</t>
+        </is>
+      </c>
+      <c r="D1470" t="inlineStr">
+        <is>
+          <t>CSE(CS)</t>
+        </is>
+      </c>
+      <c r="E1470" t="inlineStr">
+        <is>
+          <t>III</t>
+        </is>
+      </c>
+      <c r="F1470" t="inlineStr">
+        <is>
+          <t>2024 - 2028</t>
+        </is>
+      </c>
+      <c r="G1470" t="inlineStr">
+        <is>
+          <t>coder_cs_1469</t>
+        </is>
+      </c>
+      <c r="H1470" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1470" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1470" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1470" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1470" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1471">
+      <c r="A1471" t="n">
+        <v>1470</v>
+      </c>
+      <c r="B1471" t="inlineStr">
+        <is>
+          <t>732224AITEST</t>
+        </is>
+      </c>
+      <c r="C1471" t="inlineStr">
+        <is>
+          <t>AI Test Student</t>
+        </is>
+      </c>
+      <c r="D1471" t="inlineStr">
+        <is>
+          <t>CSE_AI_TEST</t>
+        </is>
+      </c>
+      <c r="E1471" t="inlineStr">
+        <is>
+          <t>III</t>
+        </is>
+      </c>
+      <c r="F1471" t="inlineStr">
+        <is>
+          <t>2024 - 2028</t>
+        </is>
+      </c>
+      <c r="G1471" t="inlineStr">
+        <is>
+          <t>aitest_user</t>
+        </is>
+      </c>
+      <c r="H1471" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1471" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1471" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1471" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1471" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1472">
+      <c r="A1472" t="n">
+        <v>1471</v>
+      </c>
+      <c r="B1472" t="inlineStr">
+        <is>
+          <t>732224TEST01</t>
+        </is>
+      </c>
+      <c r="C1472" t="inlineStr">
+        <is>
+          <t>OTP Test Student</t>
+        </is>
+      </c>
+      <c r="D1472" t="inlineStr">
+        <is>
+          <t>CSE_TEST</t>
+        </is>
+      </c>
+      <c r="E1472" t="inlineStr">
+        <is>
+          <t>III</t>
+        </is>
+      </c>
+      <c r="F1472" t="inlineStr">
+        <is>
+          <t>2024 - 2028</t>
+        </is>
+      </c>
+      <c r="G1472" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H1472" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1472" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1472" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1472" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1472" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1473">
+      <c r="A1473" t="n">
+        <v>1472</v>
+      </c>
+      <c r="B1473" t="inlineStr">
+        <is>
+          <t>TEST_URL_001</t>
+        </is>
+      </c>
+      <c r="C1473" t="inlineStr">
+        <is>
+          <t>Test Student 1</t>
+        </is>
+      </c>
+      <c r="D1473" t="inlineStr">
+        <is>
+          <t>CSE</t>
+        </is>
+      </c>
+      <c r="E1473" t="inlineStr">
+        <is>
+          <t>III</t>
+        </is>
+      </c>
+      <c r="F1473" t="inlineStr">
+        <is>
+          <t>2024 - 2028</t>
+        </is>
+      </c>
+      <c r="G1473" t="inlineStr">
+        <is>
+          <t>bharath_k</t>
+        </is>
+      </c>
+      <c r="H1473" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="I1473" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1473" t="inlineStr">
+        <is>
+          <t>NOT_ATTENDED</t>
+        </is>
+      </c>
+      <c r="K1473" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1473" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>